<commit_message>
add call scheduller on automation test and add bat file configuration
</commit_message>
<xml_diff>
--- a/testdata/Outlet.xlsx
+++ b/testdata/Outlet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Sales Force\Automation\stp-automation-test\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF8075A-2A07-4856-B610-271C85B05B96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10F9CE87-30D6-4C02-887E-64550221C571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C7681F3F-D0BE-43DE-AC81-0EAE175E5E0E}"/>
   </bookViews>
@@ -127,7 +127,7 @@
     <t>Pondok indah mall 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Cabang Pondok Indah </t>
+    <t>Cabang Pondok Indah</t>
   </si>
 </sst>
 </file>

</xml_diff>